<commit_message>
Add coding agent guide and refresh race 16 fantasy data
Document repository workflows and conventions in AGENTS.md. Add race 16 lineups and points, race 17 prices and budget, and refresh database inspection notebook outputs.
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64F5F30-B3E1-472C-8266-457FA009831F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA48154F-A262-490A-9D19-5145623136CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1725" windowWidth="21600" windowHeight="11055" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="46">
   <si>
     <t>year</t>
   </si>
@@ -548,31 +548,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T27"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:T29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.73046875" customWidth="1"/>
-    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.73046875" customWidth="1"/>
-    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.73046875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -634,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -758,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -820,7 +820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -882,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -1316,7 +1316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -1998,7 +1998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -2243,6 +2243,130 @@
         <v>42</v>
       </c>
       <c r="T27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>2026</v>
+      </c>
+      <c r="B28">
+        <v>86</v>
+      </c>
+      <c r="C28">
+        <v>16</v>
+      </c>
+      <c r="D28">
+        <v>30</v>
+      </c>
+      <c r="E28" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28">
+        <v>33</v>
+      </c>
+      <c r="G28" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28">
+        <v>35</v>
+      </c>
+      <c r="I28" t="s">
+        <v>42</v>
+      </c>
+      <c r="J28">
+        <v>37</v>
+      </c>
+      <c r="K28" t="s">
+        <v>28</v>
+      </c>
+      <c r="L28">
+        <v>45</v>
+      </c>
+      <c r="M28" t="s">
+        <v>31</v>
+      </c>
+      <c r="N28">
+        <v>36</v>
+      </c>
+      <c r="O28" t="s">
+        <v>38</v>
+      </c>
+      <c r="P28">
+        <v>6</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>36</v>
+      </c>
+      <c r="R28">
+        <v>35</v>
+      </c>
+      <c r="S28" t="s">
+        <v>42</v>
+      </c>
+      <c r="T28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>2026</v>
+      </c>
+      <c r="B29">
+        <v>86</v>
+      </c>
+      <c r="C29">
+        <v>16</v>
+      </c>
+      <c r="D29">
+        <v>30</v>
+      </c>
+      <c r="E29" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29">
+        <v>11</v>
+      </c>
+      <c r="G29" t="s">
+        <v>43</v>
+      </c>
+      <c r="H29">
+        <v>35</v>
+      </c>
+      <c r="I29" t="s">
+        <v>42</v>
+      </c>
+      <c r="J29">
+        <v>2</v>
+      </c>
+      <c r="K29" t="s">
+        <v>45</v>
+      </c>
+      <c r="L29">
+        <v>10</v>
+      </c>
+      <c r="M29" t="s">
+        <v>29</v>
+      </c>
+      <c r="N29">
+        <v>6</v>
+      </c>
+      <c r="O29" t="s">
+        <v>36</v>
+      </c>
+      <c r="P29">
+        <v>45</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>31</v>
+      </c>
+      <c r="R29">
+        <v>35</v>
+      </c>
+      <c r="S29" t="s">
+        <v>42</v>
+      </c>
+      <c r="T29" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
bahrain bugs complete, ready for singapore
</commit_message>
<xml_diff>
--- a/data/raw/driver_config.xlsx
+++ b/data/raw/driver_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA48154F-A262-490A-9D19-5145623136CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA454715-5F8B-43F5-BE7E-11C18929CBA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="15720" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{ED92144D-8F60-42AD-987F-414236BC5F32}"/>
   </bookViews>
   <sheets>
     <sheet name="DRIVER CONFIG" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="46">
   <si>
     <t>year</t>
   </si>
@@ -548,31 +548,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC79E166-4681-4991-9702-012F010761B9}">
-  <dimension ref="A1:T29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T33"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.73046875" customWidth="1"/>
+    <col min="6" max="6" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.73046875" customWidth="1"/>
+    <col min="8" max="8" width="10.3984375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.73046875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.86328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -634,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -696,7 +696,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -758,7 +758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -820,7 +820,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -882,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -1014,7 +1014,7 @@
         <v>76</v>
       </c>
       <c r="C8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8">
         <v>30</v>
@@ -1068,7 +1068,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>76</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D9">
         <v>30</v>
@@ -1130,7 +1130,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>77</v>
       </c>
       <c r="C10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>30</v>
@@ -1192,7 +1192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>77</v>
       </c>
       <c r="C11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>30</v>
@@ -1254,7 +1254,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>78</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D12">
         <v>30</v>
@@ -1316,7 +1316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>78</v>
       </c>
       <c r="C13">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D13">
         <v>30</v>
@@ -1378,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>79</v>
       </c>
       <c r="C14">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D14">
         <v>30</v>
@@ -1440,7 +1440,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>79</v>
       </c>
       <c r="C15">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D15">
         <v>30</v>
@@ -1502,7 +1502,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>80</v>
       </c>
       <c r="C16">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D16">
         <v>30</v>
@@ -1564,7 +1564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>80</v>
       </c>
       <c r="C17">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D17">
         <v>30</v>
@@ -1626,7 +1626,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>81</v>
       </c>
       <c r="C18">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D18">
         <v>30</v>
@@ -1688,7 +1688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>81</v>
       </c>
       <c r="C19">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D19">
         <v>30</v>
@@ -1750,7 +1750,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>82</v>
       </c>
       <c r="C20">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D20">
         <v>30</v>
@@ -1812,7 +1812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>82</v>
       </c>
       <c r="C21">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D21">
         <v>30</v>
@@ -1874,7 +1874,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>83</v>
       </c>
       <c r="C22">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D22">
         <v>30</v>
@@ -1936,7 +1936,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>83</v>
       </c>
       <c r="C23">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D23">
         <v>30</v>
@@ -1998,7 +1998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>84</v>
       </c>
       <c r="C24">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D24">
         <v>30</v>
@@ -2060,7 +2060,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>84</v>
       </c>
       <c r="C25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D25">
         <v>30</v>
@@ -2122,7 +2122,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>85</v>
       </c>
       <c r="C26">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D26">
         <v>30</v>
@@ -2184,7 +2184,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -2192,7 +2192,7 @@
         <v>85</v>
       </c>
       <c r="C27">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>30</v>
@@ -2246,7 +2246,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>2026</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>86</v>
       </c>
       <c r="C28">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D28">
         <v>30</v>
@@ -2308,7 +2308,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>2026</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>86</v>
       </c>
       <c r="C29">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D29">
         <v>30</v>
@@ -2367,6 +2367,254 @@
         <v>42</v>
       </c>
       <c r="T29" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A30">
+        <v>2026</v>
+      </c>
+      <c r="B30">
+        <v>87</v>
+      </c>
+      <c r="C30">
+        <v>15</v>
+      </c>
+      <c r="D30">
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30">
+        <v>33</v>
+      </c>
+      <c r="G30" t="s">
+        <v>24</v>
+      </c>
+      <c r="H30">
+        <v>35</v>
+      </c>
+      <c r="I30" t="s">
+        <v>42</v>
+      </c>
+      <c r="J30">
+        <v>37</v>
+      </c>
+      <c r="K30" t="s">
+        <v>28</v>
+      </c>
+      <c r="L30">
+        <v>45</v>
+      </c>
+      <c r="M30" t="s">
+        <v>31</v>
+      </c>
+      <c r="N30">
+        <v>36</v>
+      </c>
+      <c r="O30" t="s">
+        <v>38</v>
+      </c>
+      <c r="P30">
+        <v>6</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>36</v>
+      </c>
+      <c r="R30">
+        <v>35</v>
+      </c>
+      <c r="S30" t="s">
+        <v>42</v>
+      </c>
+      <c r="T30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A31">
+        <v>2026</v>
+      </c>
+      <c r="B31">
+        <v>87</v>
+      </c>
+      <c r="C31">
+        <v>15</v>
+      </c>
+      <c r="D31">
+        <v>30</v>
+      </c>
+      <c r="E31" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31">
+        <v>11</v>
+      </c>
+      <c r="G31" t="s">
+        <v>43</v>
+      </c>
+      <c r="H31">
+        <v>35</v>
+      </c>
+      <c r="I31" t="s">
+        <v>42</v>
+      </c>
+      <c r="J31">
+        <v>2</v>
+      </c>
+      <c r="K31" t="s">
+        <v>45</v>
+      </c>
+      <c r="L31">
+        <v>10</v>
+      </c>
+      <c r="M31" t="s">
+        <v>29</v>
+      </c>
+      <c r="N31">
+        <v>6</v>
+      </c>
+      <c r="O31" t="s">
+        <v>36</v>
+      </c>
+      <c r="P31">
+        <v>45</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>31</v>
+      </c>
+      <c r="R31">
+        <v>35</v>
+      </c>
+      <c r="S31" t="s">
+        <v>42</v>
+      </c>
+      <c r="T31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A32">
+        <v>2026</v>
+      </c>
+      <c r="B32">
+        <v>88</v>
+      </c>
+      <c r="C32">
+        <v>16</v>
+      </c>
+      <c r="D32">
+        <v>30</v>
+      </c>
+      <c r="E32" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32">
+        <v>33</v>
+      </c>
+      <c r="G32" t="s">
+        <v>24</v>
+      </c>
+      <c r="H32">
+        <v>35</v>
+      </c>
+      <c r="I32" t="s">
+        <v>42</v>
+      </c>
+      <c r="J32">
+        <v>37</v>
+      </c>
+      <c r="K32" t="s">
+        <v>28</v>
+      </c>
+      <c r="L32">
+        <v>45</v>
+      </c>
+      <c r="M32" t="s">
+        <v>31</v>
+      </c>
+      <c r="N32">
+        <v>36</v>
+      </c>
+      <c r="O32" t="s">
+        <v>38</v>
+      </c>
+      <c r="P32">
+        <v>6</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>36</v>
+      </c>
+      <c r="R32">
+        <v>35</v>
+      </c>
+      <c r="S32" t="s">
+        <v>42</v>
+      </c>
+      <c r="T32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.45">
+      <c r="A33">
+        <v>2026</v>
+      </c>
+      <c r="B33">
+        <v>88</v>
+      </c>
+      <c r="C33">
+        <v>16</v>
+      </c>
+      <c r="D33">
+        <v>30</v>
+      </c>
+      <c r="E33" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33">
+        <v>11</v>
+      </c>
+      <c r="G33" t="s">
+        <v>43</v>
+      </c>
+      <c r="H33">
+        <v>35</v>
+      </c>
+      <c r="I33" t="s">
+        <v>42</v>
+      </c>
+      <c r="J33">
+        <v>2</v>
+      </c>
+      <c r="K33" t="s">
+        <v>45</v>
+      </c>
+      <c r="L33">
+        <v>10</v>
+      </c>
+      <c r="M33" t="s">
+        <v>29</v>
+      </c>
+      <c r="N33">
+        <v>6</v>
+      </c>
+      <c r="O33" t="s">
+        <v>36</v>
+      </c>
+      <c r="P33">
+        <v>45</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>31</v>
+      </c>
+      <c r="R33">
+        <v>35</v>
+      </c>
+      <c r="S33" t="s">
+        <v>42</v>
+      </c>
+      <c r="T33" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>